<commit_message>
Process Meesho applied issue: contacts researched, cover draft in Gmail
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,11 +65,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -498,6 +513,57 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>e3d5de58d52fae70</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Meesho</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Deputy Manager - Business Finance</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bangalore, Karnataka</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/meesho/3a60c7e0-bf65-4695-bddc-9f21e68d235d</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Abhinav Singhal, Head of Business Finance VP — abhinav.singhal@meesho.com (pattern-guess) — linkedin.com/in/abhinav-singhal-b185b313 | Chandini Seth, Director Finance &amp; Strategy (CA herself) — chandini.seth@meesho.com (pattern-guess) — linkedin.com/in/chandini-seth-391aa4179 | Dhiresh Bansal, CFO — linkedin.com/in/dhiresh (not emailed — CC candidate if no response)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Process 11 applied/mailed issues: statuses for 7 jobs (Meesho x2, Fresha, Pocket FM, Cleartrip, Level AI, slice)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,11 @@
         <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -75,6 +80,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -547,22 +553,280 @@
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-10</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Abhinav Singhal, Head of Business Finance VP — abhinav.singhal@meesho.com (pattern-guess) — linkedin.com/in/abhinav-singhal-b185b313 | Chandini Seth, Director Finance &amp; Strategy (CA herself) — chandini.seth@meesho.com (pattern-guess) — linkedin.com/in/chandini-seth-391aa4179 | Dhiresh Bansal, CFO — linkedin.com/in/dhiresh (not emailed — CC candidate if no response)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>cover draft in Gmail</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Abhinav Singhal, Head of Business Finance VP — abhinav.singhal@meesho.com (pattern-guess) — linkedin.com/in/abhinav-singhal-b185b313 | Chandini Seth, Director Finance &amp; Strategy (CA herself) — chandini.seth@meesho.com (pattern-guess) — linkedin.com/in/chandini-seth-391aa4179 | Dhiresh Bansal, CFO — linkedin.com/in/dhiresh (not emailed — CC candidate if no response)</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
-        </is>
-      </c>
       <c r="K2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>e7c81f4b815b4612</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Meesho</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Deputy Manager - Business Finance</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>80</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/deputy-manager-business-finance-at-meesho-4417492845</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-10</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2d386657d54e1d83</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fresha</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Finance Analyst</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>83</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/fresha/d70472ef-6305-4e99-96ce-6a0da5a75b7c</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-10</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>beedb4f474854f0e</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pocket FM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>82</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/finance-business-partner-at-pocket-fm-4433944499</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>send cover mail</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3a3cdf1733c300f5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cleartrip</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Business Finance Manager</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>63</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/business-finance-manager-at-cleartrip-4436512956</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>send cover mail</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6b43ab081969c272</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Level AI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Finance Manager</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>78</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/private-investor-at-bortex-4433193875</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>send cover mail</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5b6bfc9989aeacb3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>slice</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Business Finance Executive</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>74</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/business-finance-executive-at-slice-4436355057</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>send cover mail</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Score 2026-07-11 batch (51 jobs): Swish 88 + Digantara 82 apply-today; contacts + Gmail cover drafts for Pocket FM, Cleartrip, Level AI, slice
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -690,14 +690,32 @@
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Abhilash Padival, CFO (ex-BofA, appointed 2026) — abhilash.padival@pocketfm.com (pattern-guess) | Rohan Nayak, Co-founder &amp; CEO — rohan.nayak@pocketfm.com (pattern-guess)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Hi Abhilash,
+I applied for the Finance Business Partner role in Bengaluru and wanted to write to you directly.
+I'm a newly qualified CA (CA Final cleared first attempt) with two years of Big-4 audit fieldwork at PwC across FMCG, manufacturing and a listed fintech — profitability analysis, product-mix variance models, and findings presented to senior leadership. I also built an AI-assisted data-validation workflow with directors that cut processing time 70–80%.
+Pocket FM's economics are cohort economics — content spend against listener LTV across markets — and that's the muscle I've deliberately built: my Third Wave Coffee unit-economics model (Excel + Power BI) showed stores turning EBITDA-positive by month 5 while the company only turns cash-positive around month 45. That unit-vs-portfolio gap is exactly what a finance business partner manages.
+I'd love 20 minutes to walk you through it. Resume and model: harshbelde.netlify.com.
+Harsh Belde
+harshbelde3@gmail.com · linkedin.com/in/harshbelde · +91 74066 54394</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail (id r-162858786086502596); verify guessed emails before sending</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -733,14 +751,32 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>CFO seat in transition (Aditya Agarwal stepped down Apr 2025, successor unannounced) | Manjari Singhal, Chief Growth &amp; Business Officer — manjari.singhal@cleartrip.com (pattern-guess)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Hi Manjari,
+I've applied for the Business Finance Manager opening in Bengaluru.
+I'm a newly qualified CA (CA Final cleared first attempt) with two years of Big-4 audit fieldwork at PwC. Most relevant to travel: on a ~₹11,000 Cr railway manufacturer I analysed payroll, hiring and leasing trends as leading indicators for workforce and premises forecasting — the same demand-signal thinking OTA planning runs on. On a listed fintech I flagged structural revenue erosion (EBITDA margin compressed 5.5% → 1.0%, profitability sustained by treasury income, not operations) to senior leadership.
+Why Cleartrip: travel is a thin-margin, high-volume business where business finance genuinely steers pricing and supply decisions — I want to learn that discipline where it's practised hardest.
+My Third Wave Coffee unit-economics model (store breakeven at month 5 vs company cash-positive at month 45) is at harshbelde.netlify.com. Could we set up a short conversation?
+Harsh Belde
+harshbelde3@gmail.com · linkedin.com/in/harshbelde · +91 74066 54394</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail (id r5418410282977485124); verify guessed emails before sending</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -776,14 +812,32 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Ashish Nagar, Founder &amp; CEO — ashish@thelevel.ai (pattern-guess) — linkedin.com/in/ashishnagar | Randall Boyce, VP Finance — randall@thelevel.ai (pattern-guess)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Hi Ashish, hi Randall,
+I've applied for the Finance Manager role in Bengaluru.
+I'm a newly qualified CA (CA Final cleared first attempt) with two years of Big-4 audit fieldwork at PwC — variance and margin modelling, and corporate performance analysis on a listed fintech where I flagged EBITDA margin compression from 5.5% to 1.0% masked by treasury income, presented to senior leadership. I also engineered an AI-assisted validation workflow with PwC directors that cut processing time 70–80% — I automate my own work, which felt worth mentioning to Level AI specifically.
+An early India finance seat at a Series C SaaS company is exactly the ownership I'm after. My Third Wave Coffee unit-economics model (Excel + Power BI: stores EBITDA-positive by month 5, company cash-positive only near month 45) shows how I think about unit vs portfolio economics — the SaaS analogue being CAC payback vs burn.
+Happy to walk you through the model on a short call. Resume: harshbelde.netlify.com.
+Harsh Belde
+harshbelde3@gmail.com · linkedin.com/in/harshbelde · +91 74066 54394</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail (id r3065641415917413547); verify guessed emails; NB stored job URL points to wrong listing (bortex)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -819,14 +873,32 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Sudhesh Chandrasekar, CFO (appointed 2020, per last public info) — sudhesh@sliceit.com (pattern-guess) | Rajan Bajaj, Founder &amp; MD/CEO slice SFB — rajan@sliceit.com (pattern-guess)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Hi Sudhesh,
+I've applied for the Business Finance Executive role in Bengaluru.
+I'm a newly qualified CA (CA Final cleared first attempt) with two years of Big-4 audit fieldwork at PwC. The most relevant piece: I led corporate performance analysis on a listed fintech, where I flagged structural revenue erosion — 2.1% YoY revenue growth against rising costs compressed EBITDA margin from 5.5% to 1.0%, with profitability sustained by ₹5.9 Cr of treasury income rather than operations. A lending book's economics get judged the same way.
+Why slice: the NESFB merger makes it the rare fintech where business finance sits inside a real bank's constraints — deposits, credit costs, regulatory capital — and I want to learn that early, close to the decisions.
+My Third Wave Coffee unit-economics model (store breakeven at month 5 vs company cash-positive at month 45) is at harshbelde.netlify.com. Could we find 20 minutes this week?
+Harsh Belde
+harshbelde3@gmail.com · linkedin.com/in/harshbelde · +91 74066 54394</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail (id r4552508998006620932); verify guessed emails before sending</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Track Porter application (Business Finance Manager, BLR) from LinkedIn confirmation
Applied 2026-07-11 via LinkedIn (job 4431070268). Record created with scraper
id convention; scored 72 apply_this_week (Series F unicorn, ~$1.2B val,
profitable FY25 — plain Manager title is the stretch).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -992,6 +992,49 @@
       <c r="J10" s="3" t="inlineStr"/>
       <c r="K10" s="3" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7a3256d0a2c143c6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Porter</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Business Finance Manager</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>72</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4431070268/</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>send cover mail</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Porter: contacts researched + cover draft in Gmail
Pankaj Shroff (CFO) + Sheeja Mathew (TA) — porter.in first.last pattern
guesses, flagged unverified. Draft r3812969596453403045.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -1026,13 +1026,21 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Pankaj Shroff, CFO — pankaj.shroff@porter.in (PATTERN-GUESS, verify before sending — Meesho guesses bounced); Sheeja Mathew, Talent Acquisition Manager — sheeja.mathew@porter.in (pattern-guess); Uttam Digga, Co-founder &amp; CEO (backup, no verified email)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail (draft id r3812969596453403045). Emails follow porter.in first.last pattern (~58-79% per RocketReach/LeadIQ) but are UNVERIFIED — cross-check on LinkedIn before sending. Attach resume before send (draft tool can't attach).</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cycle 2026-07-11 evening: 5 covers mailed (2 bounces), Swish applied+mailed, 13 jobs scored
- Mail sweep: Porter/Cleartrip/Level AI covers delivered; Pocket FM bounced on
  both pocketfm.com guesses (resend needed); slice partial bounce (sudhesh@
  rejected, rajan@ delivered). All logged via log-mail.
- Issues #15-19 processed and closed: Swish Business Finance Analyst (88)
  applied + mailed; Pocket FM mailed.
- Scored 13 new jobs from evening scrape: top = Digantara Finance Associate 84
  apply_today (right level at the Series B space-tech co); rest are senior MNC
  roles in SG/London, 25-56.
- Triggered scrape run 29162035144: success, 0 newer jobs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -696,9 +696,9 @@
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>mail bounced 2026-07-11 — resend!</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -757,9 +757,9 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-11</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -818,9 +818,9 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-11</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -879,9 +879,9 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>mail bounced 2026-07-11 — resend!</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1026,9 +1026,9 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>cover draft in Gmail</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-11</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1042,6 +1042,49 @@
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7e3c010e529d4c15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Swish</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Business Finance Analyst</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>88</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/business-finance-analyst-at-swish-4436822936</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>mailed 2026-07-11</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cycle 2026-07-16: score today's 39 jobs + clear a 116-job backlog (07-12 to 07-15); process Digantara x2 + Sturlite applied issues; mail sweep clean
- Today: Hiver (78, Series B SaaS) and BIT/Matrixport (72, Series C-II fintech)
  lead the new batch; WeRize, Digantara AM roles also apply-this-week tier
- Backlog: Tonbo Imaging (74, Series D defense-tech), Vegrow (74, Series C),
  DayOne (68, Series C data-center infra) surfaced as strong picks that had
  been sitting unscored since the 07-12 to 07-15 scrapes
- Digantara (both open roles) and Sturlite India: mailed issues had been
  filed before any draft existed (checked Gmail — nothing sent); processed
  as full applied-flow instead, one combined Digantara draft + one Sturlite
  draft created, all 4 stale issues closed with explanatory comments
- Gmail sweep: no new cover mails or replies since 07-11; one untracked
  LinkedIn confirmation (Corenza) flagged since we never scraped that listing
</commit_message>
<xml_diff>
--- a/tracker/applications.xlsx
+++ b/tracker/applications.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -983,13 +983,21 @@
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>send cover mail</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Sanjay Jain, Managing Director — sanjay.jain@sturlite.com (pattern-guess, low-confidence — no named finance leader found) — linkedin.com/company/sturlite</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail; weak contact research, MD only, verify before relying on it</t>
+        </is>
+      </c>
       <c r="K10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1085,6 +1093,108 @@
       <c r="I12" s="3" t="inlineStr"/>
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1bbd0fb0e59986f2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Digantara</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Business Finance - Finance Business Partner</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>82</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/business-finance-finance-business-partner-at-digantara-4438351713</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Sourav Barman, AVP Strategy &amp; Investments — sourav.barman@digantara.co.in (pattern-guess) — linkedin.com/in/sourav-barman-212055261 | Rahul Rawat, Co-founder &amp; COO — linkedin.com/in/rahul-rawat-digantara (not emailed — reserve if no response)</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>816268b8963dd95a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Digantara</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Finance Associate</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>84</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/finance-associate-at-digantara-4438348947</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Same outreach as FBP role (one combined mail to Sourav Barman covers both roles) — see 1bbd0fb0e59986f2</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>cover draft in Gmail</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>